<commit_message>
backup about to change figures
</commit_message>
<xml_diff>
--- a/AnalysisRevision/analysis_summary.xlsx
+++ b/AnalysisRevision/analysis_summary.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="25">
   <si>
     <t>mse</t>
   </si>
@@ -49,6 +49,9 @@
     <t>Baseline and Peak Fitting - Exponential Falloff (C Si and O)</t>
   </si>
   <si>
+    <t>Baseline and Peak Fitting - Exponential Falloff (C Si and O) - DoubleGauss</t>
+  </si>
+  <si>
     <t>Component Analysis - Elemental Maps (C Si and O) with Convex Minimizer</t>
   </si>
   <si>
@@ -62,6 +65,21 @@
   </si>
   <si>
     <t>Baseline and Peak Fitting with Exponential Falloff + Elemental Maps</t>
+  </si>
+  <si>
+    <t>Baseline and Peak Fitting with Exponential Falloff + Elemental Maps with Linear Regression</t>
+  </si>
+  <si>
+    <t>Baseline and Peak Fitting with Exponential Falloff + Elemental Maps with Feature Scaling</t>
+  </si>
+  <si>
+    <t>Baseline and Peak Fitting with Exponential Falloff + Elemental Maps with Linear Regression and Feature Scaling</t>
+  </si>
+  <si>
+    <t>Fully Featured Compound Method</t>
+  </si>
+  <si>
+    <t>Fully Featured Convex Endmembers</t>
   </si>
   <si>
     <t>C and Si</t>
@@ -428,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -447,7 +465,7 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2">
-        <v>0.001094846054911613</v>
+        <v>0.003998311040794253</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -458,7 +476,7 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3">
-        <v>1.22067821838404E-05</v>
+        <v>0.002735427864928872</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
@@ -467,12 +485,12 @@
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4">
-        <v>1.62463137760969E-05</v>
+        <v>0.003119391222010914</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
@@ -481,12 +499,12 @@
         <v>9</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5">
-        <v>9.062228695719338E-06</v>
+        <v>0.002307435883259372</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
@@ -495,26 +513,26 @@
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6">
-        <v>8.040576818718633E-06</v>
+        <v>0.009603943949269198</v>
       </c>
       <c r="B6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7">
-        <v>4.275031734424475E-06</v>
+        <v>0.002193641602160673</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
@@ -523,12 +541,12 @@
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8">
-        <v>0.0002114715934941261</v>
+        <v>0.001543791029188368</v>
       </c>
       <c r="B8" t="s">
         <v>5</v>
@@ -537,12 +555,12 @@
         <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9">
-        <v>0.0007518306829119979</v>
+        <v>0.01289467917548285</v>
       </c>
       <c r="B9" t="s">
         <v>5</v>
@@ -551,18 +569,87 @@
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10">
-        <v>2.446839403597148E-06</v>
+        <v>0.02258775521924793</v>
       </c>
       <c r="B10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11">
+        <v>0.001201658248901367</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12">
+        <v>0.00233353984703879</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13">
+        <v>0.001203457070393577</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14">
+        <v>0.001203457057799709</v>
+      </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15">
+        <v>0.001201658248901367</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16">
+        <v>0.002016487522038778</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>